<commit_message>
Remove Ventyx retrospective anchor case
</commit_message>
<xml_diff>
--- a/NewLogic 03.05.2026/ST_B_Single_Output_Template_v1.xlsx
+++ b/NewLogic 03.05.2026/ST_B_Single_Output_Template_v1.xlsx
@@ -4779,7 +4779,7 @@
     <row r="5" ht="79.5" customHeight="1" s="34">
       <c r="A5" s="50" t="inlineStr">
         <is>
-          <t>Composite forward-looking failure indicator for the integration's second half-year through 18-month window. Aggregates the FP3 (departure-trigger) signals from the other nine risk categories. This is the single forward-verifiable output that anchors sealed predictions (e.g. Eli Lilly / Ventyx).</t>
+          <t>Composite forward-looking failure indicator for the integration's second half-year through 18-month window. Aggregates the FP3 (departure-trigger) signals from the other nine risk categories. This is a forward-verifiable output for sealed predictions.</t>
         </is>
       </c>
     </row>
@@ -6210,7 +6210,7 @@
       </c>
       <c r="B28" s="49" t="inlineStr">
         <is>
-          <t>+___ / -___ ECS points (e.g. base 38 → delta to 57)</t>
+          <t>+___ / -___ ECS points</t>
         </is>
       </c>
       <c r="C28" s="47" t="n"/>

</xml_diff>